<commit_message>
Cambios para hacer responsivo el sitio y validacion de cedula con modulo-10
</commit_message>
<xml_diff>
--- a/assets/plantillas/carga_informacion_rea.xlsx
+++ b/assets/plantillas/carga_informacion_rea.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -128,6 +128,7 @@
     <xf numFmtId="49" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -502,7 +503,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plantilla de PreCarga Inicial — Sistema de Gestión de Protección de Datos (REA)</t>
+          <t>Plantilla de Carga de Información — Sistema de Gestión de Protección de Datos (REA)</t>
         </is>
       </c>
     </row>
@@ -530,7 +531,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>3. Guarde el archivo en formato Excel (.xlsx) y súbalo desde el menú Registro de Datos › PreCarga Inicial.</t>
+          <t>3. Guarde el archivo en formato Excel (.xlsx) y súbalo desde el menú Registro de Datos › Carga de Información.</t>
         </is>
       </c>
     </row>
@@ -640,58 +641,101 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>ADVERTENCIA IMPORTANTE</t>
+          <t>Qué comprueba el sistema antes de cargar</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
-          <t>La PreCarga Inicial ENCERA la información de la institución con la que usted esté conectado antes de cargar: borra</t>
+          <t>Cédula: exactamente 10 dígitos. Se revisan el código de provincia (01 a 24, o 30) y el dígito verificador,</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
-          <t>personas, empleados, estudiantes, proveedores y TODOS los consentimientos registrados, junto con su historial.</t>
+          <t>de modo que un número inventado o con una cifra cambiada se rechaza y se le indica cuál es el problema.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
-          <t>No se tocan los usuarios del sistema, roles y permisos, ni los catálogos de Finalidades y Tipos de Dato,</t>
+          <t>RUC: exactamente 13 dígitos, con su dígito verificador y el establecimiento (001 la matriz, 0001 en el sector público).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
-          <t>ni los disclaimers ni la configuración de correo.</t>
+          <t>Correo: debe tener la forma nombre@dominio.ext, sin espacios y con una extensión de al menos dos letras.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
-          <t>Las personas que tienen cuenta de usuario tampoco se borran, porque su cuenta depende de ellas.</t>
+          <t>Teléfono: solo números, con un + opcional al inicio, hasta 16 caracteres.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
-          <t>Tampoco se borran las personas que siguen vinculadas a otra institución de la red.</t>
+          <t>Una fila con un dato mal escrito NO se carga, y el motivo aparece en el resumen previo, con la hoja y el número de fila.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
-          <t>Use esta opción solo para poblar un sistema nuevo o para reiniciar una carga mal hecha.</t>
+          <t>El resto de las filas entra con normalidad: un error no detiene la carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>La carga NO borra nada</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>La Carga de Información es diferencial: compara cada fila con lo que ya consta, por el número de documento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Si la persona ya está registrada, se actualizan sus datos; si no está, se la da de alta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Puede volver a subir el mismo archivo las veces que necesite: no se duplica a nadie y no se pierde nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Los consentimientos ya otorgados y su historial se conservan siempre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Para dar de baja a alguien, hágalo desde su pantalla —Empleados, Estudiantes o Proveedores—: quitarlo del archivo no lo inactiva.</t>
         </is>
       </c>
     </row>
@@ -752,7 +796,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>(EJEMPLO) 0911111111</t>
+          <t>(EJEMPLO) 0911111110</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -8861,7 +8905,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>(EJEMPLO) 0912345678</t>
+          <t>(EJEMPLO) 0912345675</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -8896,7 +8940,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>(EJEMPLO) 0987654321</t>
+          <t>(EJEMPLO) 0923456784</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -19970,7 +20014,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>(EJEMPLO) 0987654321</t>
+          <t>(EJEMPLO) 0923456784</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -28055,7 +28099,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>(EJEMPLO) 0993456789001</t>
+          <t>(EJEMPLO) 0993456780001</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Se elimina validacion de modulo10 en cedulas y ruc, el pasaporte se limita entre 6 y 12 caracteres
</commit_message>
<xml_diff>
--- a/assets/plantillas/carga_informacion_rea.xlsx
+++ b/assets/plantillas/carga_informacion_rea.xlsx
@@ -650,21 +650,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cédula: exactamente 10 dígitos. Se revisan el código de provincia (01 a 24, o 30) y el dígito verificador,</t>
+          <t>Cédula: solo dígitos, exactamente 10. Se comprueba la forma, no la validez del número:</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>de modo que un número inventado o con una cifra cambiada se rechaza y se le indica cuál es el problema.</t>
+          <t>el dígito verificador no se revisa, de modo que también entran documentos antiguos o de personas extranjeras.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RUC: exactamente 13 dígitos, con su dígito verificador y el establecimiento (001 la matriz, 0001 en el sector público).</t>
+          <t>RUC: solo dígitos, exactamente 13.</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>

</xml_diff>